<commit_message>
Update identity schema and UI specs
Refresh the MOSIP master Excel files for the identity schema and UI specification. This keeps the reference data aligned with the latest schema and interface definitions.
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/ui_spec.xlsx
+++ b/mosip_master/xlsx/ui_spec.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\Workspace\SLUDI\MVP\Training\MaterData\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397A569D-0ACD-4E66-B787-C43A33F4A2CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF1B1D7-ACA0-4EDD-AA60-D55568D5A261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4008" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4385,689 +4385,691 @@
   </si>
   <si>
     <t>{
-	"identity": [
-		{
-			"id": "IDSchemaVersion",
-			"description": "ID Schema Version",
-			"type": "number",
-			"controlType": null,
-			"fieldType": "default",
-			"inputRequired": false,
-			"validators": [],
-			"required": true
-		},
-		{
-			"id": "familyName",
-			"description": "Family Name",
-			"labelName": {
-				"eng": "Family Name",
-				"sin": "පෙළපත් නාමය",
-				"tam": "குடும்பப் பெயர்"
+	"identity": {
+		"identity": [
+			{
+				"id": "IDSchemaVersion",
+				"description": "ID Schema Version",
+				"type": "number",
+				"controlType": null,
+				"fieldType": "default",
+				"inputRequired": false,
+				"validators": [],
+				"required": true
 			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{3,50})$",
-					"arguments": []
-				}
+			{
+				"id": "familyName",
+				"description": "Family Name",
+				"labelName": {
+					"eng": "Family Name",
+					"sin": "පෙළපත් නාමය",
+					"tam": "குடும்பப் பெயர்"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{3,50})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": true,
+				"alignmentGroup": "Name"
+			},
+			{
+				"id": "name",
+				"description": "Name",
+				"labelName": {
+					"eng": "Name",
+					"sin": "නම",
+					"tam": "பெயர்"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{3,50}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": true,
+				"alignmentGroup": "Name"
+			},
+			{
+				"id": "surname",
+				"description": "Surname",
+				"labelName": {
+					"eng": "Surname",
+					"sin": "වාසගම",
+					"tam": "குடும்பப்பெயர்"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{3,50}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": true,
+				"alignmentGroup": "Name"
+			},
+			{
+				"id": "gender",
+				"description": "gender",
+				"labelName": {
+					"eng": "Gender",
+					"sin": "ස්ත්‍රී පුරුෂ භාවය",
+					"tam": "பாலினம்"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "dynamic",
+				"type": "simpleType",
+				"validators": [],
+				"required": true,
+				"transliteration": false,
+				"subType": "gender",
+				"alignmentGroup": "Demographics"
+			},
+			{
+				"id": "dateOfBirth",
+				"description": "dateOfBirth",
+				"labelName": {
+					"eng": "Date of Birth",
+					"sin": "උපන් දිනය",
+					"tam": "பிறந்த தேதி"
+				},
+				"controlType": "ageDate",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "string",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": false,
+				"alignmentGroup": "Demographics"
+			},
+			{
+				"id": "placeOfBirth",
+				"description": "placeOfBirth",
+				"labelName": {
+					"eng": "Place of Birth",
+					"sin": "උපන් ස්ථානය",
+					"tam": "பிறந்த இடம்"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{2,128}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": true,
+				"alignmentGroup": "Demographics"
+			},
+			{
+				"id": "divisionalSecretariatOfBirth",
+				"description": "divisionalSecretariatOfBirth",
+				"labelName": {
+					"eng": "Divisional Secretariat of Birth",
+					"sin": "උපන් ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
+					"tam": "பிறந்த பிரதேச செயலகப் பிரிவு"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{1,50}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": true,
+				"alignmentGroup": "Demographics"
+			},
+			{
+				"id": "referenceIdentityNumber",
+				"description": "referenceIdentityNumber",
+				"labelName": {
+					"eng": "Existing National ID Number",
+					"sin": "පවතින ජාතික හැඳුනුම්පත් අංකය",
+					"tam": "தற்போதைய தேசிய அடையாள அட்டை எண்"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "string",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?:\\d{9}[VXvx]|\\d{12})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Identifiers"
+			},
+			{
+				"id": "addressLine1",
+				"description": "addressLine1",
+				"labelName": {
+					"eng": "Address Line 1",
+					"sin": "පළමු ලිපින පේළිය",
+					"tam": "முகவரி வரி 1"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{1,128}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": true,
+				"alignmentGroup": "Permanent Address"
+			},
+			{
+				"id": "addressLine2",
+				"description": "addressLine2",
+				"labelName": {
+					"eng": "Address Line 2",
+					"sin": "දෙවන ලිපින පේළිය",
+					"tam": "முகவரி வரி 2"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,128})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": true,
+				"alignmentGroup": "Permanent Address"
+			},
+			{
+				"id": "addressLine3",
+				"description": "addressLine3",
+				"labelName": {
+					"eng": "Address Line 3",
+					"sin": "තෙවන ලිපින පේළිය",
+					"tam": "முகவரி வரி 3"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,128})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": true,
+				"alignmentGroup": "Permanent Address"
+			},
+			{
+				"id": "province",
+				"description": "province",
+				"labelName": {
+					"eng": "Province",
+					"sin": "පළාත",
+					"tam": "மாகாணம்"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{1,50}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": false,
+				"alignmentGroup": "Permanent Address",
+				"locationHierarchyLevel": 1,
+				"parentLocCode": "LKA"
+			},
+			{
+				"id": "district",
+				"description": "district",
+				"labelName": {
+					"eng": "District",
+					"sin": "දිස්ත්‍රික්කය",
+					"tam": "மாவட்டம்"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{1,50}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": false,
+				"alignmentGroup": "Permanent Address",
+				"locationHierarchyLevel": 2
+			},
+			{
+				"id": "divisionalSecretariat",
+				"description": "divisionalSecretariat",
+				"labelName": {
+					"eng": "Divisional Secretariat Division",
+					"sin": "ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
+					"tam": "பிரதேச செயலகப் பிரிவு"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{1,50}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": false,
+				"alignmentGroup": "Permanent Address",
+				"locationHierarchyLevel": 3
+			},
+			{
+				"id": "grammaNiladhari",
+				"description": "grammaNiladhari",
+				"labelName": {
+					"eng": "Grama Niladhari Division",
+					"sin": "ග්‍රාම නිලධාරී වසම",
+					"tam": "கிராம அலுவலர் பிரிவு"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(?=.{1,50}$).*",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": false,
+				"alignmentGroup": "Permanent Address",
+				"locationHierarchyLevel": 4
+			},
+			{
+				"id": "postalCode",
+				"description": "postalCode",
+				"labelName": {
+					"eng": "Postal Code",
+					"sin": "තැපැල් කේතය",
+					"tam": "அஞ்சல் குறியீடு"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "string",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^[0-9]{5}$",
+						"arguments": []
+					}
+				],
+				"required": true,
+				"transliteration": false,
+				"alignmentGroup": "Permanent Address"
+			},
+			{
+				"id": "currentAddressLine1",
+				"description": "currentAddressLine1",
+				"labelName": {
+					"eng": "Address Line 1",
+					"sin": "පළමු ලිපින පේළිය",
+					"tam": "முகவரி வரி 1"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,128})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": true,
+				"alignmentGroup": "Current Address"
+			},
+			{
+				"id": "currentAddressLine2",
+				"description": "currentAddressLine2",
+				"labelName": {
+					"eng": "Address Line 2",
+					"sin": "දෙවන ලිපින පේළිය",
+					"tam": "முகவரி வரி 2"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,128})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": true,
+				"alignmentGroup": "Current Address"
+			},
+			{
+				"id": "currentAddressLine3",
+				"description": "currentAddressLine3",
+				"labelName": {
+					"eng": "Address Line 3",
+					"sin": "තෙවන ලිපින පේළිය",
+					"tam": "முகவரி வரி 3"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,128})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": true,
+				"alignmentGroup": "Current Address"
+			},
+			{
+				"id": "currentProvince",
+				"description": "currentProvince",
+				"labelName": {
+					"eng": "Province",
+					"sin": "පළාත",
+					"tam": "மாகாணம்"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,50})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Current Address",
+				"locationHierarchyLevel": 1,
+				"parentLocCode": "LKA"
+			},
+			{
+				"id": "currentDistrict",
+				"description": "currentDistrict",
+				"labelName": {
+					"eng": "District",
+					"sin": "දිස්ත්‍රික්කය",
+					"tam": "மாவட்டம்"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,50})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Current Address",
+				"locationHierarchyLevel": 2
+			},
+			{
+				"id": "currentDivisionalSecretariat",
+				"description": "currentDivisionalSecretariat",
+				"labelName": {
+					"eng": "Divisional Secretariat Division",
+					"sin": "ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
+					"tam": "பிரதேச செயலகப் பிரிவு"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,50})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Current Address",
+				"locationHierarchyLevel": 3
+			},
+			{
+				"id": "currentGramaNiladhari",
+				"description": "currentGramaNiladhari",
+				"labelName": {
+					"eng": "Grama Niladhari Division",
+					"sin": "ග්‍රාම නිලධාරී වසම",
+					"tam": "கிராம அலுவலர் பிரிவு"
+				},
+				"controlType": "dropdown",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "simpleType",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(|.{1,50})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Current Address",
+				"locationHierarchyLevel": 4
+			},
+			{
+				"id": "currentPostalCode",
+				"description": "currentPostalCode",
+				"labelName": {
+					"eng": "Current Postal Code",
+					"sin": "වර්තමාන තැපැල් කේතය",
+					"tam": "தற்போதைய அஞ்சல் குறியீடு"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "string",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^$|^[0-9]{5}$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Current Address"
+			},
+			{
+				"id": "phone",
+				"description": "phone",
+				"labelName": {
+					"eng": "Phone",
+					"sin": "දුරකථන අංකය",
+					"tam": "தொலைபேசி"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "string",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^(0?7[0-9]{8})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Contact"
+			},
+			{
+				"id": "email",
+				"description": "email",
+				"labelName": {
+					"eng": "Email",
+					"sin": "විද්‍යුත් තැපෑල",
+					"tam": "மின்னஞ்சல்"
+				},
+				"controlType": "textbox",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "string",
+				"validators": [
+					{
+						"type": "regex",
+						"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",
+						"arguments": []
+					}
+				],
+				"required": false,
+				"transliteration": false,
+				"alignmentGroup": "Contact"
+			},
+			{
+				"id": "proofOfAddress",
+				"description": "proofOfAddress",
+				"labelName": {
+					"eng": "Address Proof",
+					"sin": "පදිංචිය තහවුරු කිරීමේ සහතිකය",
+					"tam": "முகவரி சான்று"
+				},
+				"controlType": "fileupload",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "documentType",
+				"validators": [],
+				"required": false,
+				"transliteration": false,
+				"subType": "POA",
+				"alignmentGroup": "Documents"
+			},
+			{
+				"id": "proofOfIdentity",
+				"description": "proofOfIdentity",
+				"labelName": {
+					"eng": "Identity Proof",
+					"sin": "අනන්‍යතා තහවුරු කිරීමේ සහතිකය",
+					"tam": "அடையாளச் சான்று"
+				},
+				"controlType": "fileupload",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "documentType",
+				"validators": [],
+				"required": false,
+				"transliteration": false,
+				"subType": "POI",
+				"alignmentGroup": "Documents"
+			},
+			{
+				"id": "proofOfDateOfBirth",
+				"description": "proofOfDateOfBirth",
+				"labelName": {
+					"eng": "Date of Birth Proof",
+					"sin": "උප්පැන්න සහතිකය",
+					"tam": "பிறந்த தேதிச் சான்று"
+				},
+				"controlType": "fileupload",
+				"inputRequired": true,
+				"fieldType": "default",
+				"type": "documentType",
+				"validators": [],
+				"required": false,
+				"transliteration": false,
+				"subType": "POB",
+				"alignmentGroup": "Documents"
+			}
+		],
+		"locationHierarchy": [
+			[
+				"province",
+				"district",
+				"divisionalSecretariat",
+				"grammaNiladhari"
 			],
-			"required": false,
-			"transliteration": true,
-			"alignmentGroup": "Name"
-		},
-		{
-			"id": "name",
-			"description": "Name",
-			"labelName": {
-				"eng": "Name",
-				"sin": "නම",
-				"tam": "பெயர்"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{3,50}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": true,
-			"alignmentGroup": "Name"
-		},
-		{
-			"id": "surname",
-			"description": "Surname",
-			"labelName": {
-				"eng": "Surname",
-				"sin": "වාසගම",
-				"tam": "குடும்பப்பெயர்"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{3,50}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": true,
-			"alignmentGroup": "Name"
-		},
-		{
-			"id": "gender",
-			"description": "gender",
-			"labelName": {
-				"eng": "Gender",
-				"sin": "ස්ත්‍රී පුරුෂ භාවය",
-				"tam": "பாலினம்"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "dynamic",
-			"type": "simpleType",
-			"validators": [],
-			"required": true,
-			"transliteration": false,
-			"subType": "gender",
-			"alignmentGroup": "Demographics"
-		},
-		{
-			"id": "dateOfBirth",
-			"description": "dateOfBirth",
-			"labelName": {
-				"eng": "Date of Birth",
-				"sin": "උපන් දිනය",
-				"tam": "பிறந்த தேதி"
-			},
-			"controlType": "ageDate",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "string",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": false,
-			"alignmentGroup": "Demographics"
-		},
-		{
-			"id": "placeOfBirth",
-			"description": "placeOfBirth",
-			"labelName": {
-				"eng": "Place of Birth",
-				"sin": "උපන් ස්ථානය",
-				"tam": "பிறந்த இடம்"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{2,128}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": true,
-			"alignmentGroup": "Demographics"
-		},
-		{
-			"id": "divisionalSecretariatOfBirth",
-			"description": "divisionalSecretariatOfBirth",
-			"labelName": {
-				"eng": "Divisional Secretariat of Birth",
-				"sin": "උපන් ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
-				"tam": "பிறந்த பிரதேச செயலகப் பிரிவு"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{1,50}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": true,
-			"alignmentGroup": "Demographics"
-		},
-		{
-			"id": "referenceIdentityNumber",
-			"description": "referenceIdentityNumber",
-			"labelName": {
-				"eng": "Existing National ID Number",
-				"sin": "පවතින ජාතික හැඳුනුම්පත් අංකය",
-				"tam": "தற்போதைய தேசிய அடையாள அட்டை எண்"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "string",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?:\\d{9}[VXvx]|\\d{12})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Identifiers"
-		},
-		{
-			"id": "addressLine1",
-			"description": "addressLine1",
-			"labelName": {
-				"eng": "Address Line 1",
-				"sin": "පළමු ලිපින පේළිය",
-				"tam": "முகவரி வரி 1"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{1,128}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": true,
-			"alignmentGroup": "Permanent Address"
-		},
-		{
-			"id": "addressLine2",
-			"description": "addressLine2",
-			"labelName": {
-				"eng": "Address Line 2",
-				"sin": "දෙවන ලිපින පේළිය",
-				"tam": "முகவரி வரி 2"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,128})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": true,
-			"alignmentGroup": "Permanent Address"
-		},
-		{
-			"id": "addressLine3",
-			"description": "addressLine3",
-			"labelName": {
-				"eng": "Address Line 3",
-				"sin": "තෙවන ලිපින පේළිය",
-				"tam": "முகவரி வரி 3"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,128})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": true,
-			"alignmentGroup": "Permanent Address"
-		},
-		{
-			"id": "province",
-			"description": "province",
-			"labelName": {
-				"eng": "Province",
-				"sin": "පළාත",
-				"tam": "மாகாணம்"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{1,50}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": false,
-			"alignmentGroup": "Permanent Address",
-			"locationHierarchyLevel": 1,
-			"parentLocCode": "LKA"
-		},
-		{
-			"id": "district",
-			"description": "district",
-			"labelName": {
-				"eng": "District",
-				"sin": "දිස්ත්‍රික්කය",
-				"tam": "மாவட்டம்"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{1,50}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": false,
-			"alignmentGroup": "Permanent Address",
-			"locationHierarchyLevel": 2
-		},
-		{
-			"id": "divisionalSecretariat",
-			"description": "divisionalSecretariat",
-			"labelName": {
-				"eng": "Divisional Secretariat Division",
-				"sin": "ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
-				"tam": "பிரதேச செயலகப் பிரிவு"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{1,50}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": false,
-			"alignmentGroup": "Permanent Address",
-			"locationHierarchyLevel": 3
-		},
-		{
-			"id": "grammaNiladhari",
-			"description": "grammaNiladhari",
-			"labelName": {
-				"eng": "Grama Niladhari Division",
-				"sin": "ග්‍රාම නිලධාරී වසම",
-				"tam": "கிராம அலுவலர் பிரிவு"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(?=.{1,50}$).*",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": false,
-			"alignmentGroup": "Permanent Address",
-			"locationHierarchyLevel": 4
-		},
-		{
-			"id": "postalCode",
-			"description": "postalCode",
-			"labelName": {
-				"eng": "Postal Code",
-				"sin": "තැපැල් කේතය",
-				"tam": "அஞ்சல் குறியீடு"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "string",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^[0-9]{5}$",
-					"arguments": []
-				}
-			],
-			"required": true,
-			"transliteration": false,
-			"alignmentGroup": "Permanent Address"
-		},
-		{
-			"id": "currentAddressLine1",
-			"description": "currentAddressLine1",
-			"labelName": {
-				"eng": "Address Line 1",
-				"sin": "පළමු ලිපින පේළිය",
-				"tam": "முகவரி வரி 1"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,128})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": true,
-			"alignmentGroup": "Current Address"
-		},
-		{
-			"id": "currentAddressLine2",
-			"description": "currentAddressLine2",
-			"labelName": {
-				"eng": "Address Line 2",
-				"sin": "දෙවන ලිපින පේළිය",
-				"tam": "முகவரி வரி 2"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,128})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": true,
-			"alignmentGroup": "Current Address"
-		},
-		{
-			"id": "currentAddressLine3",
-			"description": "currentAddressLine3",
-			"labelName": {
-				"eng": "Address Line 3",
-				"sin": "තෙවන ලිපින පේළිය",
-				"tam": "முகவரி வரி 3"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,128})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": true,
-			"alignmentGroup": "Current Address"
-		},
-		{
-			"id": "currentProvince",
-			"description": "currentProvince",
-			"labelName": {
-				"eng": "Province",
-				"sin": "පළාත",
-				"tam": "மாகாணம்"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,50})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Current Address",
-			"locationHierarchyLevel": 1,
-			"parentLocCode": "LKA"
-		},
-		{
-			"id": "currentDistrict",
-			"description": "currentDistrict",
-			"labelName": {
-				"eng": "District",
-				"sin": "දිස්ත්‍රික්කය",
-				"tam": "மாவட்டம்"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,50})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Current Address",
-			"locationHierarchyLevel": 2
-		},
-		{
-			"id": "currentDivisionalSecretariat",
-			"description": "currentDivisionalSecretariat",
-			"labelName": {
-				"eng": "Divisional Secretariat Division",
-				"sin": "ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
-				"tam": "பிரதேச செயலகப் பிரிவு"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,50})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Current Address",
-			"locationHierarchyLevel": 3
-		},
-		{
-			"id": "currentGramaNiladhari",
-			"description": "currentGramaNiladhari",
-			"labelName": {
-				"eng": "Grama Niladhari Division",
-				"sin": "ග්‍රාම නිලධාරී වසම",
-				"tam": "கிராம அலுவலர் பிரிவு"
-			},
-			"controlType": "dropdown",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "simpleType",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(|.{1,50})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Current Address",
-			"locationHierarchyLevel": 4
-		},
-		{
-			"id": "currentPostalCode",
-			"description": "currentPostalCode",
-			"labelName": {
-				"eng": "Current Postal Code",
-				"sin": "වර්තමාන තැපැල් කේතය",
-				"tam": "தற்போதைய அஞ்சல் குறியீடு"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "string",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^$|^[0-9]{5}$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Current Address"
-		},
-		{
-			"id": "phone",
-			"description": "phone",
-			"labelName": {
-				"eng": "Phone",
-				"sin": "දුරකථන අංකය",
-				"tam": "தொலைபேசி"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "string",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^(0?7[0-9]{8})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Contact"
-		},
-		{
-			"id": "email",
-			"description": "email",
-			"labelName": {
-				"eng": "Email",
-				"sin": "විද්‍යුත් තැපෑල",
-				"tam": "மின்னஞ்சல்"
-			},
-			"controlType": "textbox",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "string",
-			"validators": [
-				{
-					"type": "regex",
-					"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",
-					"arguments": []
-				}
-			],
-			"required": false,
-			"transliteration": false,
-			"alignmentGroup": "Contact"
-		},
-		{
-			"id": "proofOfAddress",
-			"description": "proofOfAddress",
-			"labelName": {
-				"eng": "Address Proof",
-				"sin": "පදිංචිය තහවුරු කිරීමේ සහතිකය",
-				"tam": "முகவரி சான்று"
-			},
-			"controlType": "fileupload",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "documentType",
-			"validators": [],
-			"required": false,
-			"transliteration": false,
-			"subType": "POA",
-			"alignmentGroup": "Documents"
-		},
-		{
-			"id": "proofOfIdentity",
-			"description": "proofOfIdentity",
-			"labelName": {
-				"eng": "Identity Proof",
-				"sin": "අනන්‍යතා තහවුරු කිරීමේ සහතිකය",
-				"tam": "அடையாளச் சான்று"
-			},
-			"controlType": "fileupload",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "documentType",
-			"validators": [],
-			"required": false,
-			"transliteration": false,
-			"subType": "POI",
-			"alignmentGroup": "Documents"
-		},
-		{
-			"id": "proofOfDateOfBirth",
-			"description": "proofOfDateOfBirth",
-			"labelName": {
-				"eng": "Date of Birth Proof",
-				"sin": "උප්පැන්න සහතිකය",
-				"tam": "பிறந்த தேதிச் சான்று"
-			},
-			"controlType": "fileupload",
-			"inputRequired": true,
-			"fieldType": "default",
-			"type": "documentType",
-			"validators": [],
-			"required": false,
-			"transliteration": false,
-			"subType": "POB",
-			"alignmentGroup": "Documents"
-		}
-	],
-	"locationHierarchy": [
-		[
-			"province",
-			"district",
-			"divisionalSecretariat",
-			"grammaNiladhari"
-		],
-		[
-			"currentProvince",
-			"currentDistrict",
-			"currentDivisionalSecretariat",
-			"currentGramaNiladhari"
+			[
+				"currentProvince",
+				"currentDistrict",
+				"currentDivisionalSecretariat",
+				"currentGramaNiladhari"
+			]
 		]
-	]
+	}
 }</t>
   </si>
 </sst>

</xml_diff>

<commit_message>
updated pre-reg ui spec
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/ui_spec.xlsx
+++ b/mosip_master/xlsx/ui_spec.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\mosip-training\sludi-mvp-dev-mosip-data\mosip_master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017A40AF-3E26-46B8-89CF-C4707889C7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41071D4C-5F25-4F66-8CE3-313B14C5CCEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2784" yWindow="3228" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3064,710 +3064,710 @@
 						"eng": "</t>
   </si>
   <si>
-    <t>{
-	"identity": {
-		"identity": [
-			{
-				"id": "IDSchemaVersion",
-				"description": "ID Schema Version",
-				"type": "number",
-				"controlType": null,
-				"fieldType": "default",
-				"inputRequired": false,
-				"validators": [],
-				"required": true
-			},
-			{
-				"id": "familyName",
-				"description": "Family Name",
-				"labelName": {
-					"eng": "Family Name",
-					"sin": "පෙළපත් නාමය",
-					"tam": "குடும்பப் பெயர்"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{3,50})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": true,
-				"alignmentGroup": "Name"
-			},
-			{
-				"id": "name",
-				"description": "Name",
-				"labelName": {
-					"eng": "Name",
-					"sin": "නම",
-					"tam": "பெயர்"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": true,
-				"alignmentGroup": "Name"
-			},
-			{
-				"id": "surname",
-				"description": "Surname",
-				"labelName": {
-					"eng": "Surname",
-					"sin": "වාසගම",
-					"tam": "குடும்பப்பெயர்"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{3,50}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": true,
-				"alignmentGroup": "Name"
-			},
-			{
-				"id": "gender",
-				"description": "gender",
-				"labelName": {
-					"eng": "Gender",
-					"sin": "ස්ත්‍රී පුරුෂ භාවය",
-					"tam": "பாலினம்"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "dynamic",
-				"type": "simpleType",
-				"validators": [],
-				"required": true,
-				"transliteration": false,
-				"subType": "gender",
-				"alignmentGroup": "Demographics"
-			},
-			{
-				"id": "dateOfBirth",
-				"description": "dateOfBirth",
-				"labelName": {
-					"eng": "Date of Birth",
-					"sin": "උපන් දිනය",
-					"tam": "பிறந்த தேதி"
-				},
-				"controlType": "ageDate",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "string",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": false,
-				"alignmentGroup": "Demographics"
-			},
-			{
-				"id": "placeOfBirth",
-				"description": "placeOfBirth",
-				"labelName": {
-					"eng": "Place of Birth",
-					"sin": "උපන් ස්ථානය",
-					"tam": "பிறந்த இடம்"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{2,128}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": true,
-				"alignmentGroup": "Demographics"
-			},
-			{
-				"id": "divisionalSecretariatOfBirth",
-				"description": "divisionalSecretariatOfBirth",
-				"labelName": {
-					"eng": "Divisional Secretariat of Birth",
-					"sin": "උපන් ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
-					"tam": "பிறந்த பிரதேச செயலகப் பிரிவு"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{1,50}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": true,
-				"alignmentGroup": "Demographics"
-			},
-			{
-				"id": "referenceIdentityNumber",
-				"description": "referenceIdentityNumber",
-				"labelName": {
-					"eng": "Existing National ID Number",
-					"sin": "පවතින ජාතික හැඳුනුම්පත් අංකය",
-					"tam": "தற்போதைய தேசிய அடையாள அட்டை எண்"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "string",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?:\\d{9}[VXvx]|\\d{12})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Identifiers"
-			},
-			{
-				"id": "addressLine1",
-				"description": "addressLine1",
-				"labelName": {
-					"eng": "Address Line 1",
-					"sin": "පළමු ලිපින පේළිය",
-					"tam": "முகவரி வரி 1"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{1,128}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": true,
-				"alignmentGroup": "Permanent Address"
-			},
-			{
-				"id": "addressLine2",
-				"description": "addressLine2",
-				"labelName": {
-					"eng": "Address Line 2",
-					"sin": "දෙවන ලිපින පේළිය",
-					"tam": "முகவரி வரி 2"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,128})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": true,
-				"alignmentGroup": "Permanent Address"
-			},
-			{
-				"id": "addressLine3",
-				"description": "addressLine3",
-				"labelName": {
-					"eng": "Address Line 3",
-					"sin": "තෙවන ලිපින පේළිය",
-					"tam": "முகவரி வரி 3"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,128})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": true,
-				"alignmentGroup": "Permanent Address"
-			},
-			{
-				"id": "province",
-				"description": "province",
-				"labelName": {
-					"eng": "Province",
-					"sin": "පළාත",
-					"tam": "மாகாணம்"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{1,50}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": false,
-				"alignmentGroup": "Permanent Address",
-				"locationHierarchyLevel": 1,
-				"parentLocCode": "LKA"
-			},
-			{
-				"id": "district",
-				"description": "district",
-				"labelName": {
-					"eng": "District",
-					"sin": "දිස්ත්‍රික්කය",
-					"tam": "மாவட்டம்"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{1,50}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": false,
-				"alignmentGroup": "Permanent Address",
-				"locationHierarchyLevel": 2
-			},
-			{
-				"id": "divisionalSecretariat",
-				"description": "divisionalSecretariat",
-				"labelName": {
-					"eng": "Divisional Secretariat Division",
-					"sin": "ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
-					"tam": "பிரதேச செயலகப் பிரிவு"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{1,50}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": false,
-				"alignmentGroup": "Permanent Address",
-				"locationHierarchyLevel": 3
-			},
-			{
-				"id": "grammaNiladhari",
-				"description": "grammaNiladhari",
-				"labelName": {
-					"eng": "Grama Niladhari Division",
-					"sin": "ග්‍රාම නිලධාරී වසම",
-					"tam": "கிராம அலுவலர் பிரிவு"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(?=.{1,50}$).*",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": false,
-				"alignmentGroup": "Permanent Address",
-				"locationHierarchyLevel": 4
-			},
-			{
-				"id": "postalCode",
-				"description": "postalCode",
-				"labelName": {
-					"eng": "Postal Code",
-					"sin": "තැපැල් කේතය",
-					"tam": "அஞ்சல் குறியீடு"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "string",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^[0-9]{5}$",
-						"arguments": []
-					}
-				],
-				"required": true,
-				"transliteration": false,
-				"alignmentGroup": "Permanent Address"
-			},
-			{
-				"id": "sameAsPermanentAddress",
-				"description": "Same as Permanent Address Checkbox",
-				"labelName": {
-					"eng": "Same as Permanent Address",
-					"sin": "ස්ථිර ලිපිනයට සමානයි",
-					"tam": "நிரந்தர முகவரிக்கு ஒத்ததாக"
-				},
-				"controlType": "checkbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "boolean",
-				"validators": [],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Current Address",
-				"changeAction": "copy&amp;disable:addressLine1=currentAddressLine1,addressLine2=currentAddressLine2,addressLine3=currentAddressLine3,province=currentProvince,district=currentDistrict,divisionalSecretariat=currentDivisionalSecretariat,grammaNiladhari=currentGramaNiladhari,postalCode=currentPostalCode"
-			},
-			{
-				"id": "currentAddressLine1",
-				"description": "currentAddressLine1",
-				"labelName": {
-					"eng": "Current Address Line 1",
-					"sin": "වත්මන් පළමු ලිපින පේළිය",
-					"tam": "தற்போதைய முகவரி வரி 1"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,128})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": true,
-				"alignmentGroup": "Current Address"
-			},
-			{
-				"id": "currentAddressLine2",
-				"description": "currentAddressLine2",
-				"labelName": {
-					"eng": "Current Address Line 2",
-					"sin": "වත්මන් දෙවන ලිපින පේළිය",
-					"tam": "தற்போதைய முகவரி வரி 2"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,128})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": true,
-				"alignmentGroup": "Current Address"
-			},
-			{
-				"id": "currentAddressLine3",
-				"description": "currentAddressLine3",
-				"labelName": {
-					"eng": "Current Address Line 3",
-					"sin": "වත්මන් තෙවන ලිපින පේළිය",
-					"tam": "தற்போதைய முகவரி வரி 3"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,128})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": true,
-				"alignmentGroup": "Current Address"
-			},
-			{
-				"id": "currentProvince",
-				"description": "currentProvince",
-				"labelName": {
-					"eng": "Current Province",
-					"sin": "වත්මන් පළාත",
-					"tam": "තற்பෝதைய மாகாணம்"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,50})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Current Address",
-				"locationHierarchyLevel": 1,
-				"parentLocCode": "LKA"
-			},
-			{
-				"id": "currentDistrict",
-				"description": "currentDistrict",
-				"labelName": {
-					"eng": "Current District",
-					"sin": "වත්මන් දිස්ත්‍රික්කය",
-					"tam": "තற்பෝதைய மாவட்டம்"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,50})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Current Address",
-				"locationHierarchyLevel": 2
-			},
-			{
-				"id": "currentDivisionalSecretariat",
-				"description": "currentDivisionalSecretariat",
-				"labelName": {
-					"eng": "Current Divisional Secretariat Division",
-					"sin": "වත්මන් ප්‍රාදේශීය ලේකම් කොට්ඨාශය",
-					"tam": "தற்போதைய பிரதேச செயலகப் பிரிவு"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,50})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Current Address",
-				"locationHierarchyLevel": 3
-			},
-			{
-				"id": "currentGramaNiladhari",
-				"description": "currentGramaNiladhari",
-				"labelName": {
-					"eng": "Current Grama Niladhari Division",
-					"sin": "වත්මන් ග්‍රාම නිලධාරී වසම",
-					"tam": "தற்போதைய கிராம அலுவலர் பிரிவு"
-				},
-				"controlType": "dropdown",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "simpleType",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(|.{1,50})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Current Address",
-				"locationHierarchyLevel": 4
-			},
-			{
-				"id": "currentPostalCode",
-				"description": "currentPostalCode",
-				"labelName": {
-					"eng": "Current Postal Code",
-					"sin": "වත්මන් තැපැල් කේතය",
-					"tam": "තற்பෝதைய அஞ்சல் குறியீடு"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "string",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^[0-9]{5}$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Current Address"
-			},
-			{
-				"id": "phone",
-				"description": "phone",
-				"labelName": {
-					"eng": "Phone",
-					"sin": "දුරකථන අංකය",
-					"tam": "தொலைபேசி"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "string",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^(0?7[0-9]{8})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Contact"
-			},
-			{
-				"id": "email",
-				"description": "email",
-				"labelName": {
-					"eng": "Email",
-					"sin": "විද්‍යුත් තැපෑල",
-					"tam": "மின்னஞ்சல்"
-				},
-				"controlType": "textbox",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "string",
-				"validators": [
-					{
-						"type": "regex",
-						"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",
-						"arguments": []
-					}
-				],
-				"required": false,
-				"transliteration": false,
-				"alignmentGroup": "Contact"
-			},
-			{
-				"id": "proofOfAddress",
-				"description": "proofOfAddress",
-				"labelName": {
-					"eng": "Address Proof",
-					"sin": "පදිංචිය තහවුරු කිරීමේ සහතිකය",
-					"tam": "முகவரி சான்று"
-				},
-				"controlType": "fileupload",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "documentType",
-				"validators": [],
-				"required": false,
-				"transliteration": false,
-				"subType": "POA",
-				"alignmentGroup": "Documents"
-			},
-			{
-				"id": "proofOfIdentity",
-				"description": "proofOfIdentity",
-				"labelName": {
-					"eng": "Identity Proof",
-					"sin": "අනන්‍යතා තහවුරු කිරීමේ සහතිකය",
-					"tam": "அடையாளச் சான்று"
-				},
-				"controlType": "fileupload",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "documentType",
-				"validators": [],
-				"required": false,
-				"transliteration": false,
-				"subType": "POI",
-				"alignmentGroup": "Documents"
-			},
-			{
-				"id": "proofOfDateOfBirth",
-				"description": "proofOfDateOfBirth",
-				"labelName": {
-					"eng": "Date of Birth Proof",
-					"sin": "උප්පැන්න සහතිකය",
-					"tam": "பிறந்த தேதிச் சான்று"
-				},
-				"controlType": "fileupload",
-				"inputRequired": true,
-				"fieldType": "default",
-				"type": "documentType",
-				"validators": [],
-				"required": false,
-				"transliteration": false,
-				"subType": "POB",
-				"alignmentGroup": "Documents"
-			}
-		],
-		"locationHierarchy": [
-			[
-				"province",
-				"district",
-				"divisionalSecretariat",
-				"grammaNiladhari"
-			],
-			[
-				"currentProvince",
-				"currentDistrict",
-				"currentDivisionalSecretariat",
-				"currentGramaNiladhari"
-			]
-		]
-	}
+    <t>{_x000D_
+	"identity": {_x000D_
+		"identity": [_x000D_
+			{_x000D_
+				"id": "IDSchemaVersion",_x000D_
+				"description": "ID Schema Version",_x000D_
+				"type": "number",_x000D_
+				"controlType": null,_x000D_
+				"fieldType": "default",_x000D_
+				"inputRequired": false,_x000D_
+				"validators": [],_x000D_
+				"required": true_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "familyName",_x000D_
+				"description": "Family Name",_x000D_
+				"labelName": {_x000D_
+					"eng": "Family Name",_x000D_
+					"sin": "පෙළපත් නාමය",_x000D_
+					"tam": "குடும்பப் பெயர்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{3,50})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Name"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "name",_x000D_
+				"description": "Name",_x000D_
+				"labelName": {_x000D_
+					"eng": "Name",_x000D_
+					"sin": "නම",_x000D_
+					"tam": "பெயர்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{3,50}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Name"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "surname",_x000D_
+				"description": "Surname",_x000D_
+				"labelName": {_x000D_
+					"eng": "Surname",_x000D_
+					"sin": "වාසගම",_x000D_
+					"tam": "குடும்பப்பெயர்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{3,50}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Name"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "gender",_x000D_
+				"description": "gender",_x000D_
+				"labelName": {_x000D_
+					"eng": "Gender",_x000D_
+					"sin": "ස්ත්‍රී පුරුෂ භාවය",_x000D_
+					"tam": "பாலினம்"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "dynamic",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [],_x000D_
+				"required": true,_x000D_
+				"transliteration": false,_x000D_
+				"subType": "gender",_x000D_
+				"alignmentGroup": "Demographics"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "dateOfBirth",_x000D_
+				"description": "dateOfBirth",_x000D_
+				"labelName": {_x000D_
+					"eng": "Date of Birth",_x000D_
+					"sin": "උපන් දිනය",_x000D_
+					"tam": "பிறந்த தேதி"_x000D_
+				},_x000D_
+				"controlType": "ageDate",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "string",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(1869|18[7-9][0-9]|19[0-9][0-9]|20[0-9][0-9])/([0][1-9]|1[0-2])/([0][1-9]|[1-2][0-9]|3[01])$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Demographics"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "placeOfBirth",_x000D_
+				"description": "placeOfBirth",_x000D_
+				"labelName": {_x000D_
+					"eng": "Place of Birth",_x000D_
+					"sin": "උපන් ස්ථානය",_x000D_
+					"tam": "பிறந்த இடம்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{2,128}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Demographics"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "divisionalSecretariatOfBirth",_x000D_
+				"description": "divisionalSecretariatOfBirth",_x000D_
+				"labelName": {_x000D_
+					"eng": "Division",_x000D_
+					"sin": "කොට්ඨාශය",_x000D_
+					"tam": "பிறந்த பிரதேச செயலகப் பிரிவு"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{1,50}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Demographics"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "referenceIdentityNumber",_x000D_
+				"description": "referenceIdentityNumber",_x000D_
+				"labelName": {_x000D_
+					"eng": "Existing National ID Number",_x000D_
+					"sin": "පවතින ජාතික හැඳුනුම්පත් අංකය",_x000D_
+					"tam": "தற்போதைய தேசிய அடையாள அட்டை எண்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "string",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?:\\d{9}[VXvx]|\\d{12})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Identifiers"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "addressLine1",_x000D_
+				"description": "addressLine1",_x000D_
+				"labelName": {_x000D_
+					"eng": "Name or number of the House",_x000D_
+					"sin": "නිවසේ නම හෝ අංකය",_x000D_
+					"tam": "வீட்டின் பெயர் அல்லது இலக்கம்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{1,128}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Permanent Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "addressLine2",_x000D_
+				"description": "addressLine2",_x000D_
+				"labelName": {_x000D_
+					"eng": "Road/Street/Lane/Place/Garden",_x000D_
+					"sin": "පාර/වීදිය/පටුමඟ/පෙදෙස/උද්‍යානය",_x000D_
+					"tam": "வீதி/தெரு/ஒழுங்கை/இடம்/தோட்டம்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,128})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Permanent Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "addressLine3",_x000D_
+				"description": "addressLine3",_x000D_
+				"labelName": {_x000D_
+					"eng": "Village/City",_x000D_
+					"sin": "ගම/නගරය",_x000D_
+					"tam": "கிராமம்/நகரம்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,128})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Permanent Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "province",_x000D_
+				"description": "province",_x000D_
+				"labelName": {_x000D_
+					"eng": "Province",_x000D_
+					"sin": "පළාත",_x000D_
+					"tam": "மாகாணம்"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{1,50}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Permanent Address",_x000D_
+				"locationHierarchyLevel": 1,_x000D_
+				"parentLocCode": "LKA"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "district",_x000D_
+				"description": "district",_x000D_
+				"labelName": {_x000D_
+					"eng": "District",_x000D_
+					"sin": "දිස්ත්‍රික්කය",_x000D_
+					"tam": "மாவட்டம்"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{1,50}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Permanent Address",_x000D_
+				"locationHierarchyLevel": 2_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "divisionalSecretariat",_x000D_
+				"description": "divisionalSecretariat",_x000D_
+				"labelName": {_x000D_
+					"eng": "Divisional Secretariat Division",_x000D_
+					"sin": "ප්‍රාදේශීය ලේකම් කොට්ඨාශය",_x000D_
+					"tam": "பிரதேச செயலகப் பிரிவு"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{1,50}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Permanent Address",_x000D_
+				"locationHierarchyLevel": 3_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "grammaNiladhari",_x000D_
+				"description": "grammaNiladhari",_x000D_
+				"labelName": {_x000D_
+					"eng": "Grama Niladhari Division",_x000D_
+					"sin": "ග්‍රාම නිලධාරී වසම",_x000D_
+					"tam": "கிராம அலுவலர் பிரிவு"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(?=.{1,50}$).*",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Permanent Address",_x000D_
+				"locationHierarchyLevel": 4_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "postalCode",_x000D_
+				"description": "postalCode",_x000D_
+				"labelName": {_x000D_
+					"eng": "Postal Code",_x000D_
+					"sin": "තැපැල් කේතය",_x000D_
+					"tam": "அஞ்சல் குறியீடு"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "string",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^[0-9]{5}$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": true,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Permanent Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "sameAsPermanentAddress",_x000D_
+				"description": "Same as Permanent Address Checkbox",_x000D_
+				"labelName": {_x000D_
+					"eng": "Same as Permanent Address",_x000D_
+					"sin": "ස්ථිර ලිපිනයට සමානයි",_x000D_
+					"tam": "நிரந்தர முகவரிக்கு ஒத்ததாக"_x000D_
+				},_x000D_
+				"controlType": "checkbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "boolean",_x000D_
+				"validators": [],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Current Address",_x000D_
+				"changeAction": "copy&amp;disable:addressLine1=currentAddressLine1,addressLine2=currentAddressLine2,addressLine3=currentAddressLine3,province=currentProvince,district=currentDistrict,divisionalSecretariat=currentDivisionalSecretariat,grammaNiladhari=currentGramaNiladhari,postalCode=currentPostalCode"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentAddressLine1",_x000D_
+				"description": "currentAddressLine1",_x000D_
+				"labelName": {_x000D_
+					"eng": "Name or number of the House",_x000D_
+					"sin": "නිවසේ නම හෝ අංකය",_x000D_
+					"tam": "வீட்டின் பெயர் அல்லது இலக்கம்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,128})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Current Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentAddressLine2",_x000D_
+				"description": "currentAddressLine2",_x000D_
+				"labelName": {_x000D_
+					"eng": "Road/Street/Lane/Place/Garden",_x000D_
+					"sin": "පාර/වීදිය/පටුමඟ/පෙදෙස/උද්‍යානය",_x000D_
+					"tam": "வீதி/தெரு/ஒழுங்கை/இடம்/தோட்டம்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,128})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Current Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentAddressLine3",_x000D_
+				"description": "currentAddressLine3",_x000D_
+				"labelName": {_x000D_
+					"eng": "Village/City",_x000D_
+					"sin": "ගම/නගරය",_x000D_
+					"tam": "கிராமம்/நகரம்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,128})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": true,_x000D_
+				"alignmentGroup": "Current Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentProvince",_x000D_
+				"description": "currentProvince",_x000D_
+				"labelName": {_x000D_
+					"eng": "Province",_x000D_
+					"sin": "පළාත",_x000D_
+					"tam": "மாகாணம்"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,50})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Current Address",_x000D_
+				"locationHierarchyLevel": 1,_x000D_
+				"parentLocCode": "LKA"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentDistrict",_x000D_
+				"description": "currentDistrict",_x000D_
+				"labelName": {_x000D_
+					"eng": "District",_x000D_
+					"sin": "දිස්ත්‍රික්කය",_x000D_
+					"tam": "மாவட்டம்"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,50})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Current Address",_x000D_
+				"locationHierarchyLevel": 2_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentDivisionalSecretariat",_x000D_
+				"description": "currentDivisionalSecretariat",_x000D_
+				"labelName": {_x000D_
+					"eng": "Divisional Secretariat Division",_x000D_
+					"sin": "ප්‍රාදේශීය ලේකම් කොට්ඨාශය",_x000D_
+					"tam": "பிரதேச செயலகப் பிரிவு"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,50})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Current Address",_x000D_
+				"locationHierarchyLevel": 3_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentGramaNiladhari",_x000D_
+				"description": "currentGramaNiladhari",_x000D_
+				"labelName": {_x000D_
+					"eng": "Grama Niladhari Division",_x000D_
+					"sin": "ග්‍රාම නිලධාරී වසම",_x000D_
+					"tam": "கிராம அலுவலர் பிரிவு"_x000D_
+				},_x000D_
+				"controlType": "dropdown",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "simpleType",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(|.{1,50})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Current Address",_x000D_
+				"locationHierarchyLevel": 4_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "currentPostalCode",_x000D_
+				"description": "currentPostalCode",_x000D_
+				"labelName": {_x000D_
+					"eng": "Postal Code",_x000D_
+					"sin": "තැපැල් කේතය",_x000D_
+					"tam": "அஞ்சல் குறியீடு"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "string",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^[0-9]{5}$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Current Address"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "phone",_x000D_
+				"description": "phone",_x000D_
+				"labelName": {_x000D_
+					"eng": "Phone",_x000D_
+					"sin": "දුරකථන අංකය",_x000D_
+					"tam": "தொலைபேசி"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "string",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^(0?7[0-9]{8})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Contact"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "email",_x000D_
+				"description": "email",_x000D_
+				"labelName": {_x000D_
+					"eng": "Email",_x000D_
+					"sin": "විද්‍යුත් තැපෑල",_x000D_
+					"tam": "மின்னஞ்சல்"_x000D_
+				},_x000D_
+				"controlType": "textbox",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "string",_x000D_
+				"validators": [_x000D_
+					{_x000D_
+						"type": "regex",_x000D_
+						"validator": "^[A-Za-z0-9_\\-]+(\\.[A-Za-z0-9_]+)*@[A-Za-z0-9_-]+(\\.[A-Za-z0-9_]+)*(\\.[a-zA-Z]{2,})$",_x000D_
+						"arguments": []_x000D_
+					}_x000D_
+				],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"alignmentGroup": "Contact"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "proofOfAddress",_x000D_
+				"description": "proofOfAddress",_x000D_
+				"labelName": {_x000D_
+					"eng": "Address Proof",_x000D_
+					"sin": "පදිංචිය තහවුරු කිරීමේ ලේඛනය",_x000D_
+					"tam": "முகவரி சான்று"_x000D_
+				},_x000D_
+				"controlType": "fileupload",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "documentType",_x000D_
+				"validators": [],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"subType": "POA",_x000D_
+				"alignmentGroup": "Documents"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "proofOfIdentity",_x000D_
+				"description": "proofOfIdentity",_x000D_
+				"labelName": {_x000D_
+					"eng": "Identity Proof",_x000D_
+					"sin": "අනන්‍යතා තහවුරු කිරීමේ ලේඛනය",_x000D_
+					"tam": "அடையாளச் சான்று"_x000D_
+				},_x000D_
+				"controlType": "fileupload",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "documentType",_x000D_
+				"validators": [],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"subType": "POI",_x000D_
+				"alignmentGroup": "Documents"_x000D_
+			},_x000D_
+			{_x000D_
+				"id": "proofOfDateOfBirth",_x000D_
+				"description": "proofOfDateOfBirth",_x000D_
+				"labelName": {_x000D_
+					"eng": "Proof of Birth Details",_x000D_
+					"sin": "උපත තහවුරු කිරීමේ ලේඛනය",_x000D_
+					"tam": "பிறப்பு உறுதிப்படுத்தல் ஆவணம்"_x000D_
+				},_x000D_
+				"controlType": "fileupload",_x000D_
+				"inputRequired": true,_x000D_
+				"fieldType": "default",_x000D_
+				"type": "documentType",_x000D_
+				"validators": [],_x000D_
+				"required": false,_x000D_
+				"transliteration": false,_x000D_
+				"subType": "POB",_x000D_
+				"alignmentGroup": "Documents"_x000D_
+			}_x000D_
+		],_x000D_
+		"locationHierarchy": [_x000D_
+			[_x000D_
+				"province",_x000D_
+				"district",_x000D_
+				"divisionalSecretariat",_x000D_
+				"grammaNiladhari"_x000D_
+			],_x000D_
+			[_x000D_
+				"currentProvince",_x000D_
+				"currentDistrict",_x000D_
+				"currentDivisionalSecretariat",_x000D_
+				"currentGramaNiladhari"_x000D_
+			]_x000D_
+		]_x000D_
+	}_x000D_
 }</t>
   </si>
 </sst>

</xml_diff>